<commit_message>
Added codebook parser, unknowntype rules, fixed row prov bug, updated tests, made parsing more forgiving
</commit_message>
<xml_diff>
--- a/SDD-Validation/SDD_Validation/testData/dd_multipleVars.xlsx
+++ b/SDD-Validation/SDD_Validation/testData/dd_multipleVars.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10212"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10514"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mjohnson/Projects/SDD-Dataset/SDD-Validation/SDD_Validation/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCECBCE4-B1D1-1142-B755-06F589E53AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B2F3085-ABA7-0041-810D-30F781D30415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21500" yWindow="-8440" windowWidth="21080" windowHeight="25440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="1860" windowWidth="51200" windowHeight="30100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions " sheetId="5" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="96">
   <si>
     <t xml:space="preserve">VARNAME </t>
   </si>
@@ -270,6 +270,48 @@
   </si>
   <si>
     <t>0= bmi&lt;18.5</t>
+  </si>
+  <si>
+    <t>CODES</t>
+  </si>
+  <si>
+    <t>DEFINITION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCALE: 1=continuous, 2=categorical 3 =ordinal </t>
+  </si>
+  <si>
+    <t>COMMENT</t>
+  </si>
+  <si>
+    <t>Derived variable? 1=yes, 2=no</t>
+  </si>
+  <si>
+    <t>If derived, list source variables</t>
+  </si>
+  <si>
+    <t>If derived, provide algorithm for creating variable</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>education</t>
+  </si>
+  <si>
+    <t>educat</t>
+  </si>
+  <si>
+    <t>Cord blood arsenic level</t>
+  </si>
+  <si>
+    <t>cat</t>
   </si>
 </sst>
 </file>
@@ -463,7 +505,17 @@
     <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -488,9 +540,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -528,9 +580,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -563,26 +615,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -615,26 +650,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1307,7 +1325,7 @@
         <v>39</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>18</v>
+        <v>95</v>
       </c>
       <c r="H18" s="30" t="s">
         <v>46</v>
@@ -1324,7 +1342,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I100"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="29.33203125" style="6" customWidth="1"/>
@@ -1340,218 +1358,401 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="30.75" customHeight="1">
-      <c r="A1" s="4"/>
-      <c r="B1" s="5"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-    </row>
-    <row r="2" spans="1:9" ht="15">
-      <c r="A2"/>
-      <c r="B2" s="25"/>
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="H1" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" s="23" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="16">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>66</v>
+      </c>
       <c r="C2" s="25"/>
       <c r="E2"/>
+      <c r="G2" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H2" s="25"/>
     </row>
-    <row r="3" spans="1:9" ht="15">
-      <c r="A3"/>
-      <c r="B3" s="2"/>
+    <row r="3" spans="1:9" ht="32">
+      <c r="A3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="C3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H3" s="25"/>
     </row>
-    <row r="4" spans="1:9" ht="15">
-      <c r="A4"/>
-      <c r="B4" s="25"/>
+    <row r="4" spans="1:9" ht="32">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>21</v>
+      </c>
       <c r="C4" s="25"/>
-      <c r="E4"/>
-      <c r="H4" s="25"/>
-    </row>
-    <row r="5" spans="1:9" ht="15">
-      <c r="A5"/>
-      <c r="B5" s="25"/>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H4" s="25" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="16">
+      <c r="A5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>23</v>
+      </c>
       <c r="C5" s="25"/>
-      <c r="E5"/>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H5" s="25"/>
     </row>
-    <row r="6" spans="1:9" ht="15">
-      <c r="A6"/>
-      <c r="B6" s="25"/>
+    <row r="6" spans="1:9" ht="16">
+      <c r="A6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>51</v>
+      </c>
       <c r="C6" s="25"/>
-      <c r="E6"/>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H6" s="25"/>
     </row>
-    <row r="7" spans="1:9" ht="15">
-      <c r="A7"/>
-      <c r="B7" s="25"/>
+    <row r="7" spans="1:9" ht="16">
+      <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>27</v>
+      </c>
       <c r="C7" s="25"/>
-      <c r="E7"/>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H7" s="25"/>
     </row>
-    <row r="8" spans="1:9" ht="15">
-      <c r="A8"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
+    <row r="8" spans="1:9" ht="32">
+      <c r="A8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>59</v>
+      </c>
       <c r="D8" s="12"/>
-      <c r="E8" s="25"/>
-      <c r="H8" s="25"/>
-    </row>
-    <row r="9" spans="1:9" ht="15">
-      <c r="A9"/>
-      <c r="B9" s="25"/>
+      <c r="E8" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="16">
+      <c r="A9" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>49</v>
+      </c>
       <c r="C9" s="25"/>
       <c r="D9" s="12"/>
-      <c r="E9"/>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H9" s="25"/>
     </row>
-    <row r="10" spans="1:9" ht="15">
-      <c r="A10"/>
-      <c r="B10" s="25"/>
+    <row r="10" spans="1:9" ht="16">
+      <c r="A10" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>50</v>
+      </c>
       <c r="C10" s="25"/>
       <c r="D10" s="12"/>
-      <c r="E10"/>
+      <c r="E10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H10" s="25"/>
     </row>
-    <row r="11" spans="1:9" ht="15">
-      <c r="A11"/>
-      <c r="B11" s="25"/>
+    <row r="11" spans="1:9" ht="32">
+      <c r="A11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>48</v>
+      </c>
       <c r="C11" s="25"/>
       <c r="D11" s="12"/>
-      <c r="E11"/>
-      <c r="H11" s="25"/>
-    </row>
-    <row r="12" spans="1:9" ht="15">
-      <c r="A12"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="112">
+      <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>54</v>
+      </c>
       <c r="D12" s="12"/>
-      <c r="E12" s="25"/>
+      <c r="E12" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H12" s="25"/>
     </row>
-    <row r="13" spans="1:9" ht="15">
-      <c r="A13"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="28"/>
+    <row r="13" spans="1:9" ht="96">
+      <c r="A13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>57</v>
+      </c>
       <c r="D13" s="12"/>
-      <c r="E13" s="25"/>
-      <c r="H13" s="25"/>
-    </row>
-    <row r="14" spans="1:9" ht="15">
-      <c r="A14"/>
-      <c r="B14" s="25"/>
+      <c r="E13" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" s="25" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="16">
+      <c r="A14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>94</v>
+      </c>
       <c r="C14" s="25"/>
       <c r="D14" s="12"/>
-      <c r="E14"/>
+      <c r="E14" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H14" s="25"/>
     </row>
-    <row r="15" spans="1:9" ht="15">
-      <c r="A15"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
+    <row r="15" spans="1:9" ht="16">
+      <c r="A15" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>58</v>
+      </c>
       <c r="D15" s="12"/>
-      <c r="E15"/>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="H15" s="25"/>
     </row>
-    <row r="16" spans="1:9" customFormat="1" ht="15">
-      <c r="B16" s="3"/>
-      <c r="C16" s="29"/>
+    <row r="16" spans="1:9" customFormat="1" ht="16">
+      <c r="A16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="30" t="s">
+        <v>46</v>
+      </c>
       <c r="D16" s="25"/>
+      <c r="E16" s="25" t="s">
+        <v>18</v>
+      </c>
       <c r="F16" s="25"/>
-    </row>
-    <row r="17" spans="1:6" customFormat="1" ht="15">
-      <c r="B17" s="25"/>
-      <c r="C17" s="30"/>
+      <c r="G16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" customFormat="1" ht="16">
+      <c r="A17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="30" t="s">
+        <v>46</v>
+      </c>
       <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
+      <c r="E17" s="25" t="s">
+        <v>18</v>
+      </c>
       <c r="F17" s="25"/>
-    </row>
-    <row r="18" spans="1:6" customFormat="1" ht="15">
-      <c r="B18" s="3"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="8"/>
+      <c r="G17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="8"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="13"/>
+    </row>
+    <row r="19" spans="1:7" ht="15">
+      <c r="A19"/>
       <c r="B19" s="10"/>
       <c r="C19" s="13"/>
     </row>
-    <row r="20" spans="1:6" ht="15">
+    <row r="20" spans="1:7" ht="15">
       <c r="A20"/>
       <c r="B20" s="10"/>
       <c r="C20" s="13"/>
     </row>
-    <row r="21" spans="1:6" ht="15">
+    <row r="21" spans="1:7" ht="15">
       <c r="A21"/>
       <c r="B21" s="10"/>
       <c r="C21" s="13"/>
     </row>
-    <row r="22" spans="1:6" ht="15">
+    <row r="22" spans="1:7" ht="15">
       <c r="A22"/>
       <c r="B22" s="10"/>
       <c r="C22" s="13"/>
     </row>
-    <row r="23" spans="1:6" ht="15">
+    <row r="23" spans="1:7" ht="15">
       <c r="A23"/>
       <c r="B23" s="10"/>
       <c r="C23" s="13"/>
     </row>
-    <row r="24" spans="1:6" ht="15">
+    <row r="24" spans="1:7" ht="15">
       <c r="A24"/>
       <c r="B24" s="10"/>
       <c r="C24" s="13"/>
     </row>
-    <row r="25" spans="1:6" ht="15">
+    <row r="25" spans="1:7" ht="15">
       <c r="A25"/>
       <c r="B25" s="10"/>
-      <c r="C25" s="13"/>
-    </row>
-    <row r="26" spans="1:6" ht="15">
+      <c r="C25" s="11"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+    </row>
+    <row r="26" spans="1:7" ht="15">
       <c r="A26"/>
       <c r="B26" s="10"/>
       <c r="C26" s="11"/>
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
     </row>
-    <row r="27" spans="1:6" ht="15">
+    <row r="27" spans="1:7" ht="15">
       <c r="A27"/>
       <c r="B27" s="10"/>
       <c r="C27" s="11"/>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
     </row>
-    <row r="28" spans="1:6" ht="15">
+    <row r="28" spans="1:7" ht="15">
       <c r="A28"/>
       <c r="B28" s="10"/>
       <c r="C28" s="11"/>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
     </row>
-    <row r="29" spans="1:6" ht="15">
+    <row r="29" spans="1:7" ht="15">
       <c r="A29"/>
       <c r="B29" s="10"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-    </row>
-    <row r="30" spans="1:6" ht="15">
+      <c r="C29" s="10"/>
+    </row>
+    <row r="30" spans="1:7" ht="15">
       <c r="A30"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-    </row>
-    <row r="31" spans="1:6" ht="15">
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+    </row>
+    <row r="31" spans="1:7" ht="15">
       <c r="A31"/>
       <c r="C31" s="15"/>
       <c r="D31" s="16"/>
       <c r="E31" s="16"/>
       <c r="F31" s="16"/>
     </row>
-    <row r="32" spans="1:6" ht="15">
+    <row r="32" spans="1:7" ht="15">
       <c r="A32"/>
       <c r="C32" s="15"/>
       <c r="D32" s="16"/>
@@ -1570,14 +1771,14 @@
       <c r="C34" s="15"/>
       <c r="D34" s="16"/>
       <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
+      <c r="F34" s="17"/>
     </row>
     <row r="35" spans="1:6" ht="15">
       <c r="A35"/>
       <c r="C35" s="15"/>
       <c r="D35" s="16"/>
       <c r="E35" s="16"/>
-      <c r="F35" s="17"/>
+      <c r="F35" s="16"/>
     </row>
     <row r="36" spans="1:6" ht="15">
       <c r="A36"/>
@@ -1628,8 +1829,7 @@
       <c r="E42" s="16"/>
       <c r="F42" s="16"/>
     </row>
-    <row r="43" spans="1:6" ht="15">
-      <c r="A43"/>
+    <row r="43" spans="1:6">
       <c r="C43" s="15"/>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
@@ -1756,10 +1956,9 @@
       <c r="F63" s="16"/>
     </row>
     <row r="64" spans="3:6">
-      <c r="C64" s="15"/>
-      <c r="D64" s="16"/>
-      <c r="E64" s="16"/>
-      <c r="F64" s="16"/>
+      <c r="C64" s="18"/>
+      <c r="D64" s="19"/>
+      <c r="E64" s="19"/>
     </row>
     <row r="65" spans="3:5">
       <c r="C65" s="18"/>
@@ -1853,13 +2052,13 @@
     </row>
     <row r="83" spans="3:5">
       <c r="C83" s="18"/>
-      <c r="D83" s="19"/>
-      <c r="E83" s="19"/>
+      <c r="D83" s="20"/>
+      <c r="E83" s="20"/>
     </row>
     <row r="84" spans="3:5">
       <c r="C84" s="18"/>
-      <c r="D84" s="20"/>
-      <c r="E84" s="20"/>
+      <c r="D84" s="19"/>
+      <c r="E84" s="19"/>
     </row>
     <row r="85" spans="3:5">
       <c r="C85" s="18"/>
@@ -1936,14 +2135,12 @@
       <c r="D99" s="19"/>
       <c r="E99" s="19"/>
     </row>
-    <row r="100" spans="3:5">
-      <c r="C100" s="18"/>
-      <c r="D100" s="19"/>
-      <c r="E100" s="19"/>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  <conditionalFormatting sqref="A20:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A19">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>